<commit_message>
Outputs & scirpts for instructors
</commit_message>
<xml_diff>
--- a/output/learner_integrated_phase4A_4D/learner_phase5_integrated_phase4A_4D_results_DRAFT.xlsx
+++ b/output/learner_integrated_phase4A_4D/learner_phase5_integrated_phase4A_4D_results_DRAFT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangpinyi\Desktop\Lastinger\assessment-feedback-analysis\output\learner_integrated_phase4A_4D\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{773DAD3B-EF68-4D08-8497-6E7D0FBB9AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE085D33-4962-47AE-91ED-A61F89A0D46E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="60" windowWidth="38640" windowHeight="21120" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="60" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Workbook Guide" sheetId="1" r:id="rId1"/>
@@ -1406,13 +1406,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1424,36 +1433,462 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+  <dxfs count="149">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1642,147 +2077,147 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="tblphase4adecision" displayName="tblphase4adecision" ref="A44:B59" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="tblphase4adecision" displayName="tblphase4adecision" ref="A44:B59" totalsRowShown="0" headerRowDxfId="113" dataDxfId="112">
   <autoFilter ref="A44:B59" xr:uid="{00000000-0009-0000-0100-00000C000000}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="feature"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="result"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="feature" dataDxfId="111"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="result" dataDxfId="110"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="tblphase4bheadline" displayName="tblphase4bheadline" ref="A2:C7" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="tblphase4bheadline" displayName="tblphase4bheadline" ref="A2:C7" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
   <autoFilter ref="A2:C7" xr:uid="{00000000-0009-0000-0100-00000D000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="finding"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="evidence"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="interpretation"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="finding" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="evidence" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="interpretation" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="tblphase4bmodelfit" displayName="tblphase4bmodelfit" ref="A11:I12" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="tblphase4bmodelfit" displayName="tblphase4bmodelfit" ref="A11:I12" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <autoFilter ref="A11:I12" xr:uid="{00000000-0009-0000-0100-00000E000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="selected_model"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="analytic_n"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="number_of_parameters"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="log_likelihood"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="AIC"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="BIC"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0B00-000007000000}" name="maximum_absolute_gradient"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0B00-000008000000}" name="hessian_condition_number"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0B00-000009000000}" name="link"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="selected_model" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="analytic_n" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="number_of_parameters" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="log_likelihood" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="AIC" dataDxfId="40"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="BIC" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0B00-000007000000}" name="maximum_absolute_gradient" dataDxfId="38"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0B00-000008000000}" name="hessian_condition_number" dataDxfId="37"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0B00-000009000000}" name="link" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{00000000-000C-0000-FFFF-FFFF0C000000}" name="tblphase4beffects" displayName="tblphase4beffects" ref="A16:I20" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{00000000-000C-0000-FFFF-FFFF0C000000}" name="tblphase4beffects" displayName="tblphase4beffects" ref="A16:I20" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="A16:I20" xr:uid="{00000000-0009-0000-0100-00000F000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0C00-000001000000}" name="effect"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0C00-000002000000}" name="effect_type"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0C00-000003000000}" name="estimate"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0C00-000004000000}" name="standard_error"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0C00-000005000000}" name="z_value"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0C00-000006000000}" name="p_value"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0C00-000007000000}" name="p_value_display"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0C00-000008000000}" name="confidence_low"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0C00-000009000000}" name="confidence_high"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0C00-000001000000}" name="effect" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0C00-000002000000}" name="effect_type" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0C00-000003000000}" name="estimate" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0C00-000004000000}" name="standard_error" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0C00-000005000000}" name="z_value" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0C00-000006000000}" name="p_value" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0C00-000007000000}" name="p_value_display" dataDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0C00-000008000000}" name="confidence_low" dataDxfId="26"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0C00-000009000000}" name="confidence_high" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{00000000-000C-0000-FFFF-FFFF0D000000}" name="tblphase4bawarenessprob" displayName="tblphase4bawarenessprob" ref="A24:F27" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{00000000-000C-0000-FFFF-FFFF0D000000}" name="tblphase4bawarenessprob" displayName="tblphase4bawarenessprob" ref="A24:F27" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="A24:F27" xr:uid="{00000000-0009-0000-0100-000010000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0D00-000001000000}" name="ai_awareness_score"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0D00-000002000000}" name="ai_awareness"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0D00-000003000000}" name="predicted_probability"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0D00-000004000000}" name="standard_error"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0D00-000005000000}" name="confidence_low"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0D00-000006000000}" name="confidence_high"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0D00-000001000000}" name="ai_awareness_score" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0D00-000002000000}" name="ai_awareness" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0D00-000003000000}" name="predicted_probability" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0D00-000004000000}" name="standard_error" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0D00-000005000000}" name="confidence_low" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0D00-000006000000}" name="confidence_high" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{00000000-000C-0000-FFFF-FFFF0E000000}" name="tblphase4bfeedbackprob" displayName="tblphase4bfeedbackprob" ref="A31:I46" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{00000000-000C-0000-FFFF-FFFF0E000000}" name="tblphase4bfeedbackprob" displayName="tblphase4bfeedbackprob" ref="A31:I46" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="A31:I46" xr:uid="{00000000-0009-0000-0100-000011000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0E00-000001000000}" name="feedback_experience_half_point"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0E00-000002000000}" name="ai_awareness_score"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0E00-000003000000}" name="predicted_probability"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0E00-000004000000}" name="SE"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0E00-000005000000}" name="df"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0E00-000006000000}" name="confidence_low"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0E00-000007000000}" name="confidence_high"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0E00-000008000000}" name="ai_awareness"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0E00-000009000000}" name="feedback_experience"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0E00-000001000000}" name="feedback_experience_half_point" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0E00-000002000000}" name="ai_awareness_score" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0E00-000003000000}" name="predicted_probability" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0E00-000004000000}" name="SE" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0E00-000005000000}" name="df" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0E00-000006000000}" name="confidence_low" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0E00-000007000000}" name="confidence_high" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0E00-000008000000}" name="ai_awareness" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0E00-000009000000}" name="feedback_experience" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{00000000-000C-0000-FFFF-FFFF0F000000}" name="tblphase4bdecision" displayName="tblphase4bdecision" ref="A50:B65" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{00000000-000C-0000-FFFF-FFFF0F000000}" name="tblphase4bdecision" displayName="tblphase4bdecision" ref="A50:B65" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
   <autoFilter ref="A50:B65" xr:uid="{00000000-0009-0000-0100-000012000000}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0F00-000001000000}" name="feature"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0F00-000002000000}" name="result"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0F00-000001000000}" name="feature" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0F00-000002000000}" name="result" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{00000000-000C-0000-FFFF-FFFF10000000}" name="tblphase4cheadline" displayName="tblphase4cheadline" ref="A2:C7" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{00000000-000C-0000-FFFF-FFFF10000000}" name="tblphase4cheadline" displayName="tblphase4cheadline" ref="A2:C7" totalsRowShown="0" headerRowDxfId="109" dataDxfId="108">
   <autoFilter ref="A2:C7" xr:uid="{00000000-0009-0000-0100-000013000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1000-000001000000}" name="finding"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1000-000002000000}" name="evidence"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1000-000003000000}" name="interpretation" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1000-000001000000}" name="finding" dataDxfId="107"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1000-000002000000}" name="evidence" dataDxfId="106"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1000-000003000000}" name="interpretation" dataDxfId="105"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{00000000-000C-0000-FFFF-FFFF11000000}" name="tblphase4cdistribution" displayName="tblphase4cdistribution" ref="A11:C16" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{00000000-000C-0000-FFFF-FFFF11000000}" name="tblphase4cdistribution" displayName="tblphase4cdistribution" ref="A11:C16" totalsRowShown="0" headerRowDxfId="104" dataDxfId="103">
   <autoFilter ref="A11:C16" xr:uid="{00000000-0009-0000-0100-000014000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1100-000001000000}" name="ai_usefulness"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1100-000002000000}" name="n"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1100-000003000000}" name="percent" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1100-000001000000}" name="ai_usefulness" dataDxfId="102"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1100-000002000000}" name="n" dataDxfId="101"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1100-000003000000}" name="percent" dataDxfId="100"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{00000000-000C-0000-FFFF-FFFF12000000}" name="tblphase4cmodelfit" displayName="tblphase4cmodelfit" ref="A20:K21" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{00000000-000C-0000-FFFF-FFFF12000000}" name="tblphase4cmodelfit" displayName="tblphase4cmodelfit" ref="A20:K21" totalsRowShown="0" headerRowDxfId="99" dataDxfId="98">
   <autoFilter ref="A20:K21" xr:uid="{00000000-0009-0000-0100-000015000000}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1200-000001000000}" name="model"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1200-000002000000}" name="n"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1200-000003000000}" name="number_of_parameters" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1200-000004000000}" name="log_likelihood"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1200-000005000000}" name="AIC"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1200-000006000000}" name="BIC"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1200-000007000000}" name="convergence_code"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-1200-000008000000}" name="convergence_message"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-1200-000009000000}" name="maximum_absolute_gradient"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-1200-00000A000000}" name="hessian_condition_number"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-1200-00000B000000}" name="link"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1200-000001000000}" name="model" dataDxfId="97"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1200-000002000000}" name="n" dataDxfId="96"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1200-000003000000}" name="number_of_parameters" dataDxfId="95"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1200-000004000000}" name="log_likelihood" dataDxfId="94"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1200-000005000000}" name="AIC" dataDxfId="93"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1200-000006000000}" name="BIC" dataDxfId="92"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1200-000007000000}" name="convergence_code" dataDxfId="91"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-1200-000008000000}" name="convergence_message" dataDxfId="90"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-1200-000009000000}" name="maximum_absolute_gradient" dataDxfId="89"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-1200-00000A000000}" name="hessian_condition_number" dataDxfId="88"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-1200-00000B000000}" name="link" dataDxfId="87"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1803,65 +2238,65 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{00000000-000C-0000-FFFF-FFFF13000000}" name="tblphase4ceffects" displayName="tblphase4ceffects" ref="A25:G27" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{00000000-000C-0000-FFFF-FFFF13000000}" name="tblphase4ceffects" displayName="tblphase4ceffects" ref="A25:G27" totalsRowShown="0" headerRowDxfId="86" dataDxfId="85">
   <autoFilter ref="A25:G27" xr:uid="{00000000-0009-0000-0100-000016000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1300-000001000000}" name="effect"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1300-000002000000}" name="effect_type"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1300-000003000000}" name="estimate" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1300-000004000000}" name="standard_error"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1300-000005000000}" name="z_value"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1300-000006000000}" name="p_value"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1300-000007000000}" name="p_value_display"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1300-000001000000}" name="effect" dataDxfId="84"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1300-000002000000}" name="effect_type" dataDxfId="83"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1300-000003000000}" name="estimate" dataDxfId="82"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1300-000004000000}" name="standard_error" dataDxfId="81"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1300-000005000000}" name="z_value" dataDxfId="80"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1300-000006000000}" name="p_value" dataDxfId="79"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1300-000007000000}" name="p_value_display" dataDxfId="78"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{00000000-000C-0000-FFFF-FFFF14000000}" name="tblphase4cpredictedprob" displayName="tblphase4cpredictedprob" ref="A31:J36" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{00000000-000C-0000-FFFF-FFFF14000000}" name="tblphase4cpredictedprob" displayName="tblphase4cpredictedprob" ref="A31:J36" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
   <autoFilter ref="A31:J36" xr:uid="{00000000-0009-0000-0100-000017000000}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1400-000001000000}" name="ai_comfort_score"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1400-000002000000}" name="ai_comfort"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1400-000003000000}" name="predicted_probability" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1400-000004000000}" name="standard_error"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1400-000005000000}" name="confidence_low_raw"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1400-000006000000}" name="confidence_high_raw"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1400-000007000000}" name="confidence_low"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-1400-000008000000}" name="confidence_high"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-1400-000009000000}" name="label_y"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-1400-00000A000000}" name="percent_label"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1400-000001000000}" name="ai_comfort_score" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1400-000002000000}" name="ai_comfort" dataDxfId="74"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1400-000003000000}" name="predicted_probability" dataDxfId="73"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1400-000004000000}" name="standard_error" dataDxfId="72"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1400-000005000000}" name="confidence_low_raw" dataDxfId="71"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1400-000006000000}" name="confidence_high_raw" dataDxfId="70"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1400-000007000000}" name="confidence_low" dataDxfId="69"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-1400-000008000000}" name="confidence_high" dataDxfId="68"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-1400-000009000000}" name="label_y" dataDxfId="67"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-1400-00000A000000}" name="percent_label" dataDxfId="66"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{00000000-000C-0000-FFFF-FFFF15000000}" name="tblphase4clocationscale" displayName="tblphase4clocationscale" ref="A40:F42" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{00000000-000C-0000-FFFF-FFFF15000000}" name="tblphase4clocationscale" displayName="tblphase4clocationscale" ref="A40:F42" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
   <autoFilter ref="A40:F42" xr:uid="{00000000-0009-0000-0100-000018000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1500-000001000000}" name="no.par"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1500-000002000000}" name="AIC"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1500-000003000000}" name="logLik" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1500-000004000000}" name="LR.stat"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1500-000005000000}" name="df"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1500-000006000000}" name="Pr(&gt;Chisq)"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1500-000001000000}" name="no.par" dataDxfId="63"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1500-000002000000}" name="AIC" dataDxfId="62"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1500-000003000000}" name="logLik" dataDxfId="61"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1500-000004000000}" name="LR.stat" dataDxfId="60"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1500-000005000000}" name="df" dataDxfId="59"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1500-000006000000}" name="Pr(&gt;Chisq)" dataDxfId="58"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{00000000-000C-0000-FFFF-FFFF16000000}" name="tblphase4cfeedbackadd" displayName="tblphase4cfeedbackadd" ref="A46:F48" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{00000000-000C-0000-FFFF-FFFF16000000}" name="tblphase4cfeedbackadd" displayName="tblphase4cfeedbackadd" ref="A46:F48" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
   <autoFilter ref="A46:F48" xr:uid="{00000000-0009-0000-0100-000019000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1600-000001000000}" name="no.par"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1600-000002000000}" name="AIC"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1600-000003000000}" name="logLik" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1600-000004000000}" name="LR.stat"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1600-000005000000}" name="df"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1600-000006000000}" name="Pr(&gt;Chisq)"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1600-000001000000}" name="no.par" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1600-000002000000}" name="AIC" dataDxfId="54"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1600-000003000000}" name="logLik" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1600-000004000000}" name="LR.stat" dataDxfId="52"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1600-000005000000}" name="df" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1600-000006000000}" name="Pr(&gt;Chisq)" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2052,70 +2487,70 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="tblphase4aheadline" displayName="tblphase4aheadline" ref="A2:D12" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="tblphase4aheadline" displayName="tblphase4aheadline" ref="A2:D12" totalsRowShown="0" headerRowDxfId="148" dataDxfId="147">
   <autoFilter ref="A2:D12" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="result"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="estimate"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="interpretation"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="reporting_caution"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="result" dataDxfId="146"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="estimate" dataDxfId="145"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="interpretation" dataDxfId="144"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="reporting_caution" dataDxfId="143"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblphase4apolychoric" displayName="tblphase4apolychoric" ref="A16:E20" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblphase4apolychoric" displayName="tblphase4apolychoric" ref="A16:E20" totalsRowShown="0" headerRowDxfId="142" dataDxfId="141">
   <autoFilter ref="A16:E20" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="row"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="rubric_clear_aligned"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="feedback_specific_relevant"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="feedback_helped_improve"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="feedback_timely"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="row" dataDxfId="140"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="rubric_clear_aligned" dataDxfId="139"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="feedback_specific_relevant" dataDxfId="138"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="feedback_helped_improve" dataDxfId="137"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="feedback_timely" dataDxfId="136"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblphase4aordinalitems" displayName="tblphase4aordinalitems" ref="A24:C28" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblphase4aordinalitems" displayName="tblphase4aordinalitems" ref="A24:C28" totalsRowShown="0" headerRowDxfId="135" dataDxfId="134">
   <autoFilter ref="A24:C28" xr:uid="{00000000-0009-0000-0100-000009000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="item"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="ordinal_item_rest_correlation"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="ordinal_alpha_if_deleted"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="item" dataDxfId="133"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="ordinal_item_rest_correlation" dataDxfId="132"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="ordinal_alpha_if_deleted" dataDxfId="131"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblphase4aobservedreliability" displayName="tblphase4aobservedreliability" ref="A32:E34" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblphase4aobservedreliability" displayName="tblphase4aobservedreliability" ref="A32:E34" totalsRowShown="0" headerRowDxfId="130" dataDxfId="129">
   <autoFilter ref="A32:E34" xr:uid="{00000000-0009-0000-0100-00000A000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="composite"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="number_of_items"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="raw_alpha"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="standardized_alpha"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="average_pearson_correlation"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="composite" dataDxfId="128"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="number_of_items" dataDxfId="127"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="raw_alpha" dataDxfId="126"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="standardized_alpha" dataDxfId="125"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="average_pearson_correlation" dataDxfId="124"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="tblphase4acomposite" displayName="tblphase4acomposite" ref="A38:H40" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="tblphase4acomposite" displayName="tblphase4acomposite" ref="A38:H40" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
   <autoFilter ref="A38:H40" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="composite"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="valid_n"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="mean"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="standard_deviation"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="minimum"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="maximum"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="maximum_score_n"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="maximum_score_percent"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="composite" dataDxfId="121"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="valid_n" dataDxfId="120"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="mean" dataDxfId="119"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="standard_deviation" dataDxfId="118"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="minimum" dataDxfId="117"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="maximum" dataDxfId="116"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="maximum_score_n" dataDxfId="115"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="maximum_score_percent" dataDxfId="114"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2412,22 +2847,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -2567,14 +3002,14 @@
     <col min="5" max="5" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" ht="24" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>407</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -2806,23 +3241,23 @@
     <col min="4" max="5" width="66.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" ht="24" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
     </row>
     <row r="2" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -2937,23 +3372,23 @@
     <col min="5" max="5" width="61.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" ht="24" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -3069,16 +3504,16 @@
     <col min="7" max="7" width="58.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -3618,600 +4053,601 @@
   <dimension ref="A1:H59"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.7109375" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <col min="3" max="4" width="28.7109375" customWidth="1"/>
-    <col min="5" max="10" width="24.7109375" customWidth="1"/>
+    <col min="1" max="1" width="42.7109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" style="3" customWidth="1"/>
+    <col min="3" max="4" width="28.7109375" style="3" customWidth="1"/>
+    <col min="5" max="10" width="24.7109375" style="3" customWidth="1"/>
+    <col min="11" max="16384" width="11.42578125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D3" s="1"/>
+      <c r="D3" s="4"/>
     </row>
     <row r="4" spans="1:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D4" s="1"/>
+      <c r="D4" s="4"/>
     </row>
     <row r="5" spans="1:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D5" s="1"/>
+      <c r="D5" s="4"/>
     </row>
     <row r="6" spans="1:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="1"/>
+      <c r="D6" s="4"/>
     </row>
     <row r="7" spans="1:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="D7" s="1"/>
+      <c r="D7" s="4"/>
     </row>
     <row r="8" spans="1:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D8" s="1"/>
+      <c r="D8" s="4"/>
     </row>
     <row r="9" spans="1:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="4" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="D11" s="1"/>
+      <c r="D11" s="4"/>
     </row>
     <row r="12" spans="1:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="4" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="3" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17" s="4">
         <v>1</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="4">
         <v>0.79751847331386305</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="4">
         <v>0.699283935466114</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="4">
         <v>0.52358960364957796</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="4">
         <v>0.79751847331386305</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18" s="4">
         <v>1</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="4">
         <v>0.90061272937644798</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="4">
         <v>0.68608809456450903</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19" s="4">
         <v>0.699283935466114</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" s="4">
         <v>0.90061272937644798</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="4">
         <v>1</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="4">
         <v>0.59680666568888097</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="4">
         <v>0.52358960364957796</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="4">
         <v>0.68608809456450903</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="4">
         <v>0.59680666568888097</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="A24" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="3" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B25" s="4">
         <v>0.74437172216787195</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" s="4">
         <v>0.88916915295152399</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26" s="4">
         <v>0.92530109583880904</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26" s="4">
         <v>0.82222387061754498</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+      <c r="A27" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B27" s="4">
         <v>0.82942358674226602</v>
       </c>
-      <c r="C27" s="1">
+      <c r="C27" s="4">
         <v>0.858461890935584</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+      <c r="A28" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="B28" s="1">
+      <c r="B28" s="4">
         <v>0.64703962100244805</v>
       </c>
-      <c r="C28" s="1">
+      <c r="C28" s="4">
         <v>0.92269429346335796</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="A32" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="3" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
+      <c r="A33" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="B33" s="1">
+      <c r="B33" s="4">
         <v>4</v>
       </c>
-      <c r="C33" s="1">
+      <c r="C33" s="4">
         <v>0.78087321885275796</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="4">
         <v>0.79975789206654102</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="4">
         <v>0.49962187800334901</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
+      <c r="A34" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="B34" s="1">
+      <c r="B34" s="4">
         <v>3</v>
       </c>
-      <c r="C34" s="1">
+      <c r="C34" s="4">
         <v>0.63137085315376595</v>
       </c>
-      <c r="D34" s="1">
+      <c r="D34" s="4">
         <v>0.65599866019424002</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="4">
         <v>0.38862418177275199</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="B37" s="6"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="A38" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E38" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F38" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="G38" t="s">
+      <c r="G38" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="H38" t="s">
+      <c r="H38" s="3" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
+      <c r="A39" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="B39" s="1">
+      <c r="B39" s="4">
         <v>170</v>
       </c>
-      <c r="C39" s="1">
+      <c r="C39" s="4">
         <v>4.8</v>
       </c>
-      <c r="D39" s="1">
+      <c r="D39" s="4">
         <v>0.43650033720341902</v>
       </c>
-      <c r="E39" s="1">
+      <c r="E39" s="4">
         <v>2.25</v>
       </c>
-      <c r="F39" s="1">
+      <c r="F39" s="4">
         <v>5</v>
       </c>
-      <c r="G39" s="1">
+      <c r="G39" s="4">
         <v>121</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="4">
         <v>71.176470588235304</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
+      <c r="A40" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="B40" s="1">
+      <c r="B40" s="4">
         <v>170</v>
       </c>
-      <c r="C40" s="1">
+      <c r="C40" s="4">
         <v>4.7901960784313697</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="4">
         <v>0.433365907724587</v>
       </c>
-      <c r="E40" s="1">
+      <c r="E40" s="4">
         <v>2.3333333333333299</v>
       </c>
-      <c r="F40" s="1">
+      <c r="F40" s="4">
         <v>5</v>
       </c>
-      <c r="G40" s="1">
+      <c r="G40" s="4">
         <v>121</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="4">
         <v>71.176470588235304</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
+      <c r="A43" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="B43" s="6"/>
-      <c r="C43" s="6"/>
-      <c r="D43" s="6"/>
+      <c r="B43" s="9"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+      <c r="A44" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="3" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
+      <c r="A45" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" s="4" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
+      <c r="A46" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" s="4" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
+      <c r="A47" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" s="4" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
+      <c r="A48" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" s="4" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
+      <c r="A49" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" s="4" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
+      <c r="A50" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" s="4" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
+      <c r="A51" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" s="4" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
+      <c r="A52" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" s="4" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
+      <c r="A53" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" s="4" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
+      <c r="A54" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" s="4" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
+      <c r="A55" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" s="4" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
+      <c r="A56" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" s="4" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
+      <c r="A57" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" s="4" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
+      <c r="A58" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" s="4" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
+      <c r="A59" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" s="4" t="s">
         <v>113</v>
       </c>
     </row>
@@ -4245,1015 +4681,1016 @@
   <dimension ref="A1:I65"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="48.7109375" customWidth="1"/>
-    <col min="2" max="2" width="32.7109375" customWidth="1"/>
-    <col min="3" max="3" width="41.42578125" customWidth="1"/>
-    <col min="4" max="11" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="48.7109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="41.42578125" style="3" customWidth="1"/>
+    <col min="4" max="11" width="22.7109375" style="3" customWidth="1"/>
+    <col min="12" max="16384" width="11.42578125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="4" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="4" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="4" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="4" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="3" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="4">
         <v>170</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="4">
         <v>10</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="4">
         <v>-193.16482364425499</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="4">
         <v>406.32964728850999</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12" s="4">
         <v>437.68763165901203</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="4">
         <v>3.2702876295864802E-8</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="4">
         <v>1301.31627807825</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="I12" s="4" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I16" s="3" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="4">
         <v>4.8072506699175701</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="4">
         <v>1.97850804623326</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="4">
         <v>2.4297352133946299</v>
       </c>
-      <c r="F17" s="1">
+      <c r="F17" s="4">
         <v>1.5109857088528701E-2</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="G17" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="4">
         <v>0.92944615617767201</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="4">
         <v>8.6850551836574699</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18" s="4">
         <v>1.3511782186394901</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="4">
         <v>0.36004752334816698</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="4">
         <v>3.75277742803106</v>
       </c>
-      <c r="F18" s="1">
+      <c r="F18" s="4">
         <v>1.748861191692E-4</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="4" t="s">
         <v>251</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="4">
         <v>0.64549804015423695</v>
       </c>
-      <c r="I18" s="1">
+      <c r="I18" s="4">
         <v>2.0568583971247398</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" s="4">
         <v>0.66936004761821699</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="4">
         <v>0.25433623691395002</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="4">
         <v>2.63179189776517</v>
       </c>
-      <c r="F19" s="1">
+      <c r="F19" s="4">
         <v>8.4935870229608402E-3</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="G19" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="4">
         <v>0.17087018330342699</v>
       </c>
-      <c r="I19" s="1">
+      <c r="I19" s="4">
         <v>1.1678499119330099</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="4">
         <v>0.25817098671796201</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="4">
         <v>0.119985187009894</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="4">
         <v>2.1516904974001001</v>
       </c>
-      <c r="F20" s="1">
+      <c r="F20" s="4">
         <v>3.1421739071155398E-2</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="G20" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="4">
         <v>2.30043415002672E-2</v>
       </c>
-      <c r="I20" s="1">
+      <c r="I20" s="4">
         <v>0.493337631935657</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="A24" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="3" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
+      <c r="A25" s="4">
         <v>0</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" s="4">
         <v>0.48643571979869898</v>
       </c>
-      <c r="D25" s="1">
+      <c r="D25" s="4">
         <v>7.5542580668872802E-2</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="4">
         <v>0.338374982388497</v>
       </c>
-      <c r="F25" s="1">
+      <c r="F25" s="4">
         <v>0.63449645720890202</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
+      <c r="A26" s="4">
         <v>1</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26" s="4">
         <v>0.71754824601539002</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="4">
         <v>3.9724378260617602E-2</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="4">
         <v>0.63968989531633402</v>
       </c>
-      <c r="F26" s="1">
+      <c r="F26" s="4">
         <v>0.79540659671444702</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
+      <c r="A27" s="4">
         <v>2</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="C27" s="1">
+      <c r="C27" s="4">
         <v>0.82185610966455103</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="4">
         <v>3.3584291281325201E-2</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="4">
         <v>0.75603210830685097</v>
       </c>
-      <c r="F27" s="1">
+      <c r="F27" s="4">
         <v>0.88768011102225097</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="A31" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="H31" t="s">
+      <c r="H31" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="I31" t="s">
+      <c r="I31" s="3" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1">
+      <c r="A32" s="4">
         <v>-1.6</v>
       </c>
-      <c r="B32" s="1">
+      <c r="B32" s="4">
         <v>0</v>
       </c>
-      <c r="C32" s="1">
+      <c r="C32" s="4">
         <v>0.28730994304539598</v>
       </c>
-      <c r="D32" s="1">
+      <c r="D32" s="4">
         <v>8.2049349124095006E-2</v>
       </c>
-      <c r="E32" s="1" t="e">
+      <c r="E32" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F32" s="1">
+      <c r="F32" s="4">
         <v>0.12649617380721601</v>
       </c>
-      <c r="G32" s="1">
+      <c r="G32" s="4">
         <v>0.448123712283575</v>
       </c>
-      <c r="H32" s="1" t="s">
+      <c r="H32" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="I32" s="1">
+      <c r="I32" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="1">
+      <c r="A33" s="4">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="B33" s="1">
+      <c r="B33" s="4">
         <v>0</v>
       </c>
-      <c r="C33" s="1">
+      <c r="C33" s="4">
         <v>0.34235309229204203</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="4">
         <v>7.9802758198717197E-2</v>
       </c>
-      <c r="E33" s="1" t="e">
+      <c r="E33" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F33" s="1">
+      <c r="F33" s="4">
         <v>0.185942560355598</v>
       </c>
-      <c r="G33" s="1">
+      <c r="G33" s="4">
         <v>0.49876362422848602</v>
       </c>
-      <c r="H33" s="1" t="s">
+      <c r="H33" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="I33" s="1">
+      <c r="I33" s="4">
         <v>4.25</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
+      <c r="A34" s="4">
         <v>-0.6</v>
       </c>
-      <c r="B34" s="1">
+      <c r="B34" s="4">
         <v>0</v>
       </c>
-      <c r="C34" s="1">
+      <c r="C34" s="4">
         <v>0.40461421545854198</v>
       </c>
-      <c r="D34" s="1">
+      <c r="D34" s="4">
         <v>7.6384026227907506E-2</v>
       </c>
-      <c r="E34" s="1" t="e">
+      <c r="E34" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F34" s="1">
+      <c r="F34" s="4">
         <v>0.25490427505768098</v>
       </c>
-      <c r="G34" s="1">
+      <c r="G34" s="4">
         <v>0.55432415585940398</v>
       </c>
-      <c r="H34" s="1" t="s">
+      <c r="H34" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="I34" s="1">
+      <c r="I34" s="4">
         <v>4.5</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
+      <c r="A35" s="4">
         <v>-9.9999999999999603E-2</v>
       </c>
-      <c r="B35" s="1">
+      <c r="B35" s="4">
         <v>0</v>
       </c>
-      <c r="C35" s="1">
+      <c r="C35" s="4">
         <v>0.472417077245325</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="4">
         <v>7.5199196320309594E-2</v>
       </c>
-      <c r="E35" s="1" t="e">
+      <c r="E35" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F35" s="1">
+      <c r="F35" s="4">
         <v>0.32502936079116201</v>
       </c>
-      <c r="G35" s="1">
+      <c r="G35" s="4">
         <v>0.61980479369948904</v>
       </c>
-      <c r="H35" s="1" t="s">
+      <c r="H35" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="I35" s="1">
+      <c r="I35" s="4">
         <v>4.75</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
+      <c r="A36" s="4">
         <v>0.4</v>
       </c>
-      <c r="B36" s="1">
+      <c r="B36" s="4">
         <v>0</v>
       </c>
-      <c r="C36" s="1">
+      <c r="C36" s="4">
         <v>0.54328007762816</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="4">
         <v>7.9227419334642404E-2</v>
       </c>
-      <c r="E36" s="1" t="e">
+      <c r="E36" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F36" s="1">
+      <c r="F36" s="4">
         <v>0.387997189144208</v>
       </c>
-      <c r="G36" s="1">
+      <c r="G36" s="4">
         <v>0.69856296611211099</v>
       </c>
-      <c r="H36" s="1" t="s">
+      <c r="H36" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="I36" s="1">
+      <c r="I36" s="4">
         <v>5</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="1">
+      <c r="A37" s="4">
         <v>-1.6</v>
       </c>
-      <c r="B37" s="1">
+      <c r="B37" s="4">
         <v>1</v>
       </c>
-      <c r="C37" s="1">
+      <c r="C37" s="4">
         <v>0.54412154607822205</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="4">
         <v>7.5024492594474607E-2</v>
       </c>
-      <c r="E37" s="1" t="e">
+      <c r="E37" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F37" s="1">
+      <c r="F37" s="4">
         <v>0.39707624263466001</v>
       </c>
-      <c r="G37" s="1">
+      <c r="G37" s="4">
         <v>0.69116684952178398</v>
       </c>
-      <c r="H37" s="1" t="s">
+      <c r="H37" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="I37" s="1">
+      <c r="I37" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
+      <c r="A38" s="4">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="B38" s="1">
+      <c r="B38" s="4">
         <v>1</v>
       </c>
-      <c r="C38" s="1">
+      <c r="C38" s="4">
         <v>0.60087741913360304</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="4">
         <v>5.9425357182765599E-2</v>
       </c>
-      <c r="E38" s="1" t="e">
+      <c r="E38" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F38" s="1">
+      <c r="F38" s="4">
         <v>0.48440585928695401</v>
       </c>
-      <c r="G38" s="1">
+      <c r="G38" s="4">
         <v>0.71734897898025296</v>
       </c>
-      <c r="H38" s="1" t="s">
+      <c r="H38" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="I38" s="1">
+      <c r="I38" s="4">
         <v>4.25</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="1">
+      <c r="A39" s="4">
         <v>-0.6</v>
       </c>
-      <c r="B39" s="1">
+      <c r="B39" s="4">
         <v>1</v>
       </c>
-      <c r="C39" s="1">
+      <c r="C39" s="4">
         <v>0.65587113683320097</v>
       </c>
-      <c r="D39" s="1">
+      <c r="D39" s="4">
         <v>4.6831987396521703E-2</v>
       </c>
-      <c r="E39" s="1" t="e">
+      <c r="E39" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F39" s="1">
+      <c r="F39" s="4">
         <v>0.56408212821158499</v>
       </c>
-      <c r="G39" s="1">
+      <c r="G39" s="4">
         <v>0.74766014545481796</v>
       </c>
-      <c r="H39" s="1" t="s">
+      <c r="H39" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="I39" s="1">
+      <c r="I39" s="4">
         <v>4.5</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="1">
+      <c r="A40" s="4">
         <v>-9.9999999999999603E-2</v>
       </c>
-      <c r="B40" s="1">
+      <c r="B40" s="4">
         <v>1</v>
       </c>
-      <c r="C40" s="1">
+      <c r="C40" s="4">
         <v>0.70767574395690602</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="4">
         <v>4.02166036320298E-2</v>
       </c>
-      <c r="E40" s="1" t="e">
+      <c r="E40" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F40" s="1">
+      <c r="F40" s="4">
         <v>0.62885264925760498</v>
       </c>
-      <c r="G40" s="1">
+      <c r="G40" s="4">
         <v>0.78649883865620696</v>
       </c>
-      <c r="H40" s="1" t="s">
+      <c r="H40" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="I40" s="1">
+      <c r="I40" s="4">
         <v>4.75</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="1">
+      <c r="A41" s="4">
         <v>0.4</v>
       </c>
-      <c r="B41" s="1">
+      <c r="B41" s="4">
         <v>1</v>
       </c>
-      <c r="C41" s="1">
+      <c r="C41" s="4">
         <v>0.75516298084495403</v>
       </c>
-      <c r="D41" s="1">
+      <c r="D41" s="4">
         <v>3.9989601134209102E-2</v>
       </c>
-      <c r="E41" s="1" t="e">
+      <c r="E41" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F41" s="1">
+      <c r="F41" s="4">
         <v>0.67678480286578302</v>
       </c>
-      <c r="G41" s="1">
+      <c r="G41" s="4">
         <v>0.83354115882412605</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="H41" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="I41" s="1">
+      <c r="I41" s="4">
         <v>5</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="1">
+      <c r="A42" s="4">
         <v>-1.6</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="4">
         <v>2</v>
       </c>
-      <c r="C42" s="1">
+      <c r="C42" s="4">
         <v>0.71421620254240403</v>
       </c>
-      <c r="D42" s="1">
+      <c r="D42" s="4">
         <v>5.8159738685878197E-2</v>
       </c>
-      <c r="E42" s="1" t="e">
+      <c r="E42" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F42" s="1">
+      <c r="F42" s="4">
         <v>0.60022520936782198</v>
       </c>
-      <c r="G42" s="1">
+      <c r="G42" s="4">
         <v>0.82820719571698598</v>
       </c>
-      <c r="H42" s="1" t="s">
+      <c r="H42" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="I42" s="1">
+      <c r="I42" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="1">
+      <c r="A43" s="4">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="B43" s="1">
+      <c r="B43" s="4">
         <v>2</v>
       </c>
-      <c r="C43" s="1">
+      <c r="C43" s="4">
         <v>0.75141232181092699</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="4">
         <v>4.6606836355161697E-2</v>
       </c>
-      <c r="E43" s="1" t="e">
+      <c r="E43" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F43" s="1">
+      <c r="F43" s="4">
         <v>0.66006460112145804</v>
       </c>
-      <c r="G43" s="1">
+      <c r="G43" s="4">
         <v>0.84276004250039604</v>
       </c>
-      <c r="H43" s="1" t="s">
+      <c r="H43" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="I43" s="1">
+      <c r="I43" s="4">
         <v>4.25</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="1">
+      <c r="A44" s="4">
         <v>-0.6</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="4">
         <v>2</v>
       </c>
-      <c r="C44" s="1">
+      <c r="C44" s="4">
         <v>0.78544036541420603</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="4">
         <v>3.8524571566717902E-2</v>
       </c>
-      <c r="E44" s="1" t="e">
+      <c r="E44" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F44" s="1">
+      <c r="F44" s="4">
         <v>0.709933592623603</v>
       </c>
-      <c r="G44" s="1">
+      <c r="G44" s="4">
         <v>0.86094713820480895</v>
       </c>
-      <c r="H44" s="1" t="s">
+      <c r="H44" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="I44" s="1">
+      <c r="I44" s="4">
         <v>4.5</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="1">
+      <c r="A45" s="4">
         <v>-9.9999999999999603E-2</v>
       </c>
-      <c r="B45" s="1">
+      <c r="B45" s="4">
         <v>2</v>
       </c>
-      <c r="C45" s="1">
+      <c r="C45" s="4">
         <v>0.81612544831427802</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="4">
         <v>3.40878822530611E-2</v>
       </c>
-      <c r="E45" s="1" t="e">
+      <c r="E45" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F45" s="1">
+      <c r="F45" s="4">
         <v>0.74931442678903604</v>
       </c>
-      <c r="G45" s="1">
+      <c r="G45" s="4">
         <v>0.88293646983951901</v>
       </c>
-      <c r="H45" s="1" t="s">
+      <c r="H45" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="I45" s="1">
+      <c r="I45" s="4">
         <v>4.75</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="1">
+      <c r="A46" s="4">
         <v>0.4</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="4">
         <v>2</v>
       </c>
-      <c r="C46" s="1">
+      <c r="C46" s="4">
         <v>0.84343403499943803</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="4">
         <v>3.25105317671684E-2</v>
       </c>
-      <c r="E46" s="1" t="e">
+      <c r="E46" s="4" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="F46" s="1">
+      <c r="F46" s="4">
         <v>0.77971456361754299</v>
       </c>
-      <c r="G46" s="1">
+      <c r="G46" s="4">
         <v>0.90715350638133396</v>
       </c>
-      <c r="H46" s="1" t="s">
+      <c r="H46" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="I46" s="1">
+      <c r="I46" s="4">
         <v>5</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="6" t="s">
+      <c r="A49" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="B49" s="6"/>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
+      <c r="B49" s="9"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+      <c r="A50" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="3" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
+      <c r="A51" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" s="4" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
+      <c r="A52" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" s="4" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
+      <c r="A53" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" s="4" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
+      <c r="A54" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" s="4" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
+      <c r="A55" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" s="4" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
+      <c r="A56" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" s="4" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
+      <c r="A57" s="4" t="s">
         <v>281</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" s="4" t="s">
         <v>282</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
+      <c r="A58" s="4" t="s">
         <v>283</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" s="4" t="s">
         <v>284</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
+      <c r="A59" s="4" t="s">
         <v>285</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" s="4" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
+      <c r="A60" s="4" t="s">
         <v>287</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B60" s="4" t="s">
         <v>288</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="1" t="s">
+      <c r="A61" s="4" t="s">
         <v>289</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" s="4" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="1" t="s">
+      <c r="A62" s="4" t="s">
         <v>291</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B62" s="4" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="1" t="s">
+      <c r="A63" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B63" s="4" t="s">
         <v>294</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="1" t="s">
+      <c r="A64" s="4" t="s">
         <v>295</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B64" s="4" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="1" t="s">
+      <c r="A65" s="4" t="s">
         <v>297</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="B65" s="4" t="s">
         <v>298</v>
       </c>
     </row>
@@ -5287,656 +5724,657 @@
   <dimension ref="A1:K48"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.7109375" customWidth="1"/>
-    <col min="2" max="2" width="42" customWidth="1"/>
-    <col min="3" max="3" width="34" style="7" customWidth="1"/>
-    <col min="4" max="11" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="45.7109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="42" style="3" customWidth="1"/>
+    <col min="3" max="3" width="34" style="5" customWidth="1"/>
+    <col min="4" max="11" width="22.7109375" style="3" customWidth="1"/>
+    <col min="12" max="16384" width="11.42578125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="9" t="s">
         <v>299</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="5" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="4" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="4" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="4" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="4" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="9" t="s">
         <v>300</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="5" t="s">
         <v>303</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="4" t="s">
         <v>304</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="4">
         <v>7</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="4">
         <v>4.1176470588235299</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="4" t="s">
         <v>305</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="4">
         <v>20</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="4">
         <v>11.764705882352899</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="4" t="s">
         <v>306</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="4">
         <v>26</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="4">
         <v>15.294117647058799</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="4" t="s">
         <v>307</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15" s="4">
         <v>55</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="4">
         <v>32.352941176470601</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="4" t="s">
         <v>308</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16" s="4">
         <v>62</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="4">
         <v>36.470588235294102</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="A20" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="I20" t="s">
+      <c r="I20" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="K20" t="s">
+      <c r="K20" s="3" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="4" t="s">
         <v>312</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21" s="4">
         <v>170</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21" s="4">
         <v>10</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="4">
         <v>-169.61435196904</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="4">
         <v>359.22870393808103</v>
       </c>
-      <c r="F21" s="1">
+      <c r="F21" s="4">
         <v>390.58668830858301</v>
       </c>
-      <c r="G21" s="1">
+      <c r="G21" s="4">
         <v>0</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="H21" s="4" t="s">
         <v>313</v>
       </c>
-      <c r="I21" s="1">
+      <c r="I21" s="4">
         <v>3.2134295224750499E-12</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="4">
         <v>38408.2228436937</v>
       </c>
-      <c r="K21" s="1" t="s">
+      <c r="K21" s="4" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="9" t="s">
         <v>314</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="A25" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="3" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26" s="4">
         <v>3.6773642271081801</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="4">
         <v>1.0456686040229399</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="4">
         <v>3.51675876368523</v>
       </c>
-      <c r="F26" s="1">
+      <c r="F26" s="4">
         <v>4.36850616945304E-4</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="G26" s="4" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+      <c r="A27" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="C27" s="1">
+      <c r="C27" s="4">
         <v>0.271512289987278</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="4">
         <v>9.6388973791838806E-2</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="4">
         <v>2.8168397204189999</v>
       </c>
-      <c r="F27" s="1">
+      <c r="F27" s="4">
         <v>4.8498721855183601E-3</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="G27" s="4" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="9" t="s">
         <v>318</v>
       </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
-      <c r="J30" s="6"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="A31" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="H31" t="s">
+      <c r="H31" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="I31" t="s">
+      <c r="I31" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="J31" t="s">
+      <c r="J31" s="3" t="s">
         <v>323</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1">
+      <c r="A32" s="4">
         <v>0</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="4" t="s">
         <v>304</v>
       </c>
-      <c r="C32" s="1">
+      <c r="C32" s="4">
         <v>1.08715978052725E-2</v>
       </c>
-      <c r="D32" s="1">
+      <c r="D32" s="4">
         <v>2.8084273301759201E-2</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="4">
         <v>-4.4172566398155297E-2</v>
       </c>
-      <c r="F32" s="1">
+      <c r="F32" s="4">
         <v>6.5915762008700293E-2</v>
       </c>
-      <c r="G32" s="1">
+      <c r="G32" s="4">
         <v>0</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="4">
         <v>6.5915762008700293E-2</v>
       </c>
-      <c r="I32" s="1">
+      <c r="I32" s="4">
         <v>0.1059157620087</v>
       </c>
-      <c r="J32" s="1" t="s">
+      <c r="J32" s="4" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="1">
+      <c r="A33" s="4">
         <v>1</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="4" t="s">
         <v>305</v>
       </c>
-      <c r="C33" s="1">
+      <c r="C33" s="4">
         <v>9.6256454800200703E-2</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="4">
         <v>3.99685883663237E-2</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="4">
         <v>1.79194610892996E-2</v>
       </c>
-      <c r="F33" s="1">
+      <c r="F33" s="4">
         <v>0.17459344851110201</v>
       </c>
-      <c r="G33" s="1">
+      <c r="G33" s="4">
         <v>1.79194610892996E-2</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="4">
         <v>0.17459344851110201</v>
       </c>
-      <c r="I33" s="1">
+      <c r="I33" s="4">
         <v>0.21459344851110199</v>
       </c>
-      <c r="J33" s="1" t="s">
+      <c r="J33" s="4" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
+      <c r="A34" s="4">
         <v>2</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="4" t="s">
         <v>306</v>
       </c>
-      <c r="C34" s="1">
+      <c r="C34" s="4">
         <v>0.41824319094803902</v>
       </c>
-      <c r="D34" s="1">
+      <c r="D34" s="4">
         <v>6.2193151109490301E-2</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="4">
         <v>0.29634685468838101</v>
       </c>
-      <c r="F34" s="1">
+      <c r="F34" s="4">
         <v>0.54013952720769698</v>
       </c>
-      <c r="G34" s="1">
+      <c r="G34" s="4">
         <v>0.29634685468838101</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="4">
         <v>0.54013952720769698</v>
       </c>
-      <c r="I34" s="1">
+      <c r="I34" s="4">
         <v>0.58013952720769701</v>
       </c>
-      <c r="J34" s="1" t="s">
+      <c r="J34" s="4" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
+      <c r="A35" s="4">
         <v>3</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="4" t="s">
         <v>307</v>
       </c>
-      <c r="C35" s="1">
+      <c r="C35" s="4">
         <v>0.78664021300532605</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="4">
         <v>3.6142135187641401E-2</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="4">
         <v>0.71580292971317105</v>
       </c>
-      <c r="F35" s="1">
+      <c r="F35" s="4">
         <v>0.85747749629748105</v>
       </c>
-      <c r="G35" s="1">
+      <c r="G35" s="4">
         <v>0.71580292971317105</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="4">
         <v>0.85747749629748105</v>
       </c>
-      <c r="I35" s="1">
+      <c r="I35" s="4">
         <v>0.89747749629748097</v>
       </c>
-      <c r="J35" s="1" t="s">
+      <c r="J35" s="4" t="s">
         <v>327</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
+      <c r="A36" s="4">
         <v>4</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="4" t="s">
         <v>308</v>
       </c>
-      <c r="C36" s="1">
+      <c r="C36" s="4">
         <v>0.90383967963936096</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="4">
         <v>2.94415655543733E-2</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="4">
         <v>0.846135271504315</v>
       </c>
-      <c r="F36" s="1">
+      <c r="F36" s="4">
         <v>0.96154408777440803</v>
       </c>
-      <c r="G36" s="1">
+      <c r="G36" s="4">
         <v>0.846135271504315</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="4">
         <v>0.96154408777440803</v>
       </c>
-      <c r="I36" s="1">
+      <c r="I36" s="4">
         <v>1.00154408777441</v>
       </c>
-      <c r="J36" s="1" t="s">
+      <c r="J36" s="4" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="6" t="s">
+      <c r="A39" s="9" t="s">
         <v>329</v>
       </c>
-      <c r="B39" s="6"/>
-      <c r="C39" s="6"/>
-      <c r="D39" s="6"/>
-      <c r="E39" s="6"/>
-      <c r="F39" s="6"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="A40" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="5" t="s">
         <v>331</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E40" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="F40" t="s">
+      <c r="F40" s="3" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="1">
+      <c r="A41" s="4">
         <v>9</v>
       </c>
-      <c r="B41" s="1">
+      <c r="B41" s="4">
         <v>365.33677598408798</v>
       </c>
-      <c r="C41" s="1">
+      <c r="C41" s="4">
         <v>-173.66838799204399</v>
       </c>
-      <c r="D41" s="1"/>
-      <c r="E41" s="1"/>
-      <c r="F41" s="1"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
     </row>
     <row r="42" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="1">
+      <c r="A42" s="4">
         <v>10</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="4">
         <v>359.22870393808103</v>
       </c>
-      <c r="C42" s="1">
+      <c r="C42" s="4">
         <v>-169.61435196904</v>
       </c>
-      <c r="D42" s="1">
+      <c r="D42" s="4">
         <v>8.1080720460075195</v>
       </c>
-      <c r="E42" s="1">
+      <c r="E42" s="4">
         <v>1</v>
       </c>
-      <c r="F42" s="1">
+      <c r="F42" s="4">
         <v>4.4068572179397003E-3</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="6" t="s">
+      <c r="A45" s="9" t="s">
         <v>334</v>
       </c>
-      <c r="B45" s="6"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="6"/>
+      <c r="B45" s="9"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+      <c r="A46" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="C46" s="5" t="s">
         <v>331</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E46" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F46" s="3" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="1">
+      <c r="A47" s="4">
         <v>10</v>
       </c>
-      <c r="B47" s="1">
+      <c r="B47" s="4">
         <v>359.22870393808103</v>
       </c>
-      <c r="C47" s="1">
+      <c r="C47" s="4">
         <v>-169.61435196904</v>
       </c>
-      <c r="D47" s="1"/>
-      <c r="E47" s="1"/>
-      <c r="F47" s="1"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
     </row>
     <row r="48" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="1">
+      <c r="A48" s="4">
         <v>11</v>
       </c>
-      <c r="B48" s="1">
+      <c r="B48" s="4">
         <v>361.21789400393499</v>
       </c>
-      <c r="C48" s="1">
+      <c r="C48" s="4">
         <v>-169.608947001968</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="4">
         <v>1.0809934145072499E-2</v>
       </c>
-      <c r="E48" s="1">
+      <c r="E48" s="4">
         <v>1</v>
       </c>
-      <c r="F48" s="1">
+      <c r="F48" s="4">
         <v>0.91719249487478305</v>
       </c>
     </row>
@@ -5979,12 +6417,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="10" t="s">
         <v>335</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -6053,12 +6491,12 @@
       </c>
     </row>
     <row r="10" spans="1:4" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="10" t="s">
         <v>336</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -6131,12 +6569,12 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="10" t="s">
         <v>342</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -6279,14 +6717,14 @@
       </c>
     </row>
     <row r="31" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="10" t="s">
         <v>226</v>
       </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -6329,18 +6767,18 @@
       </c>
     </row>
     <row r="36" spans="1:10" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="6" t="s">
+      <c r="A36" s="10" t="s">
         <v>352</v>
       </c>
-      <c r="B36" s="6"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
+      <c r="J36" s="10"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
@@ -6407,18 +6845,18 @@
       </c>
     </row>
     <row r="41" spans="1:10" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
+      <c r="A41" s="10" t="s">
         <v>359</v>
       </c>
-      <c r="B41" s="6"/>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
-      <c r="E41" s="6"/>
-      <c r="F41" s="6"/>
-      <c r="G41" s="6"/>
-      <c r="H41" s="6"/>
-      <c r="I41" s="6"/>
-      <c r="J41" s="6"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
+      <c r="J41" s="10"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
@@ -6645,16 +7083,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="6" t="s">
+      <c r="A51" s="10" t="s">
         <v>365</v>
       </c>
-      <c r="B51" s="6"/>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6"/>
-      <c r="E51" s="6"/>
-      <c r="F51" s="6"/>
-      <c r="G51" s="6"/>
-      <c r="H51" s="6"/>
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="10"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
@@ -6735,14 +7173,14 @@
       </c>
     </row>
     <row r="57" spans="1:8" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="6" t="s">
+      <c r="A57" s="10" t="s">
         <v>374</v>
       </c>
-      <c r="B57" s="6"/>
-      <c r="C57" s="6"/>
-      <c r="D57" s="6"/>
-      <c r="E57" s="6"/>
-      <c r="F57" s="6"/>
+      <c r="B57" s="10"/>
+      <c r="C57" s="10"/>
+      <c r="D57" s="10"/>
+      <c r="E57" s="10"/>
+      <c r="F57" s="10"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -7065,16 +7503,16 @@
       </c>
     </row>
     <row r="76" spans="1:8" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="6" t="s">
+      <c r="A76" s="10" t="s">
         <v>395</v>
       </c>
-      <c r="B76" s="6"/>
-      <c r="C76" s="6"/>
-      <c r="D76" s="6"/>
-      <c r="E76" s="6"/>
-      <c r="F76" s="6"/>
-      <c r="G76" s="6"/>
-      <c r="H76" s="6"/>
+      <c r="B76" s="10"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="10"/>
+      <c r="E76" s="10"/>
+      <c r="F76" s="10"/>
+      <c r="G76" s="10"/>
+      <c r="H76" s="10"/>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
@@ -7297,75 +7735,75 @@
     <col min="1" max="10" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:10" ht="24" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="10" t="s">
         <v>403</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
     </row>
     <row r="35" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
+      <c r="A35" s="10" t="s">
         <v>404</v>
       </c>
-      <c r="B35" s="6"/>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
-      <c r="H35" s="6"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="6"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
+      <c r="J35" s="10"/>
     </row>
     <row r="67" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A67" s="6" t="s">
+      <c r="A67" s="10" t="s">
         <v>405</v>
       </c>
-      <c r="B67" s="6"/>
-      <c r="C67" s="6"/>
-      <c r="D67" s="6"/>
-      <c r="E67" s="6"/>
-      <c r="F67" s="6"/>
-      <c r="G67" s="6"/>
-      <c r="H67" s="6"/>
-      <c r="I67" s="6"/>
-      <c r="J67" s="6"/>
+      <c r="B67" s="10"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="10"/>
+      <c r="E67" s="10"/>
+      <c r="F67" s="10"/>
+      <c r="G67" s="10"/>
+      <c r="H67" s="10"/>
+      <c r="I67" s="10"/>
+      <c r="J67" s="10"/>
     </row>
     <row r="99" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A99" s="6" t="s">
+      <c r="A99" s="10" t="s">
         <v>406</v>
       </c>
-      <c r="B99" s="6"/>
-      <c r="C99" s="6"/>
-      <c r="D99" s="6"/>
-      <c r="E99" s="6"/>
-      <c r="F99" s="6"/>
-      <c r="G99" s="6"/>
-      <c r="H99" s="6"/>
-      <c r="I99" s="6"/>
-      <c r="J99" s="6"/>
+      <c r="B99" s="10"/>
+      <c r="C99" s="10"/>
+      <c r="D99" s="10"/>
+      <c r="E99" s="10"/>
+      <c r="F99" s="10"/>
+      <c r="G99" s="10"/>
+      <c r="H99" s="10"/>
+      <c r="I99" s="10"/>
+      <c r="J99" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>